<commit_message>
feat(closing): Japanese first — page defaults, fonts, wording and file names
This is a product for users in Japan. Found by scanning everything a Japanese user sees:
- the page was <html lang="zh-CN"> with Chinese title and Chinese fallback text; now Japanese (matches T.ja)
- only a Simplified Chinese font was loaded, so kanji rendered in Chinese glyph forms; Japanese fonts by default, Chinese fonts for the Chinese UI
- Japanese and English strings contained Chinese file names, sheet names and words; replaced
- names written into the working folder follow the language (会社資料.xlsx, 締め結果/, ワークペーパー_ja.xlsx); existing names are kept
- engine: Japanese messages cleaned of Chinese; the Japanese workpaper no longer has a Chinese account-name column; old workbook messages follow the workbook language
- tests/closing-japanese.test.mjs keeps it that way

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solutions/demo/closing-engine/template_ja.xlsx
+++ b/solutions/demo/closing-engine/template_ja.xlsx
@@ -1927,17 +1927,17 @@
     <row r="3" ht="174" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>要確認の事項の番号（画面と底稿にあります）。ふつうは自動で入ります。</t>
+          <t>要確認の事項の番号（画面とワークペーパーにあります）。ふつうは自動で入ります。</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>「記帳」＝この 1 件をどの科目に入れるかを答える。「処理済み」＝別の方法で済んでいるので、もう尋ねなくてよい。</t>
+          <t>「仕訳する」＝この 1 件をどの科目に入れるかを答える。「処理済み」＝別の方法で済んでいるので、もう尋ねなくてよい。</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
         <is>
-          <t>「記帳」のとき：相手の科目。</t>
+          <t>「仕訳する」のとき：相手の科目。</t>
         </is>
       </c>
       <c r="D3" s="6" t="inlineStr">
@@ -2044,7 +2044,7 @@
   </mergeCells>
   <dataValidations count="3">
     <dataValidation sqref="B5:B2000" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="ドロップダウンから選んでください" error="この欄は、一覧から 1 つ選びます。" type="list">
-      <formula1>"記帳,処理済み"</formula1>
+      <formula1>"仕訳する,処理済み"</formula1>
     </dataValidation>
     <dataValidation sqref="C5:C2000" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>='科目表'!$B$2:$B$400</formula1>
@@ -5899,7 +5899,7 @@
       </c>
       <c r="F3" s="6" t="inlineStr">
         <is>
-          <t>対応する中国語の科目名。空でも構いません（中日 2 言語の底稿にだけ表示）。</t>
+          <t>対応する中国語の科目名。空でも構いません（中国語と日本語を併記するワークペーパーにだけ表示）。</t>
         </is>
       </c>
     </row>
@@ -6372,7 +6372,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>底稿に表示する名前。氏名でも記号でも構いません。</t>
+          <t>ワークペーパーに表示する名前。氏名でも記号でも構いません。</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">

</xml_diff>

<commit_message>
feat(closing): Japanese in です・ます form — engine wording, page strings, guard test
Engine bundle rebuilt from d952edb (plain-form sentence endings 296 -> 0; check names are noun phrases).
Page: four Japanese strings made polite; HTML fallback kept in sync; cache-bust refreshed.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/solutions/demo/closing-engine/template_ja.xlsx
+++ b/solutions/demo/closing-engine/template_ja.xlsx
@@ -1267,7 +1267,7 @@
       <c r="A1" s="7" t="inlineStr">
         <is>
           <t>この表：毎月決まって出てくる入出金（家賃・得意先の入金・手数料…）。「摘要にこの字があれば、この科目」とあらかじめ書いておくと、1 件ずつ尋ねられなくなります。
-いつ書くか：書くことを勧めますが、必須ではありません：書かなくても締められ、明細を 1 件ずつ尋ねるだけです。給与・社会保険・源泉所得税・住民税の支払と、自社の口座どうしの振替は書かなくてよい（自動で照合します）。
+いつ書くか：書くことを勧めますが、必須ではありません：書かなくても締められ、明細を 1 件ずつ尋ねるだけです。給与・社会保険・源泉所得税・住民税の支払と、自社の口座どうしの振替は書かなくてかまいません（自動で照合します）。
 書かないと：1 つのルールには 1 つの科目だけ。1 件の入出金を 2 科目に分けるもの（借入の返済＝元金＋利息、手数料を引かれた入金、源泉所得税を天引きした報酬の支払）はルールにせず、締めた後に画面でその 1 件に「回答」して分けます。</t>
         </is>
       </c>
@@ -1932,7 +1932,7 @@
       </c>
       <c r="B3" s="6" t="inlineStr">
         <is>
-          <t>「仕訳する」＝この 1 件をどの科目に入れるかを答える。「処理済み」＝別の方法で済んでいるので、もう尋ねなくてよい。</t>
+          <t>「仕訳する」＝この 1 件をどの科目に入れるかを答えます。「処理済み」＝別の方法で済んでいるので、もう尋ねません。</t>
         </is>
       </c>
       <c r="C3" s="6" t="inlineStr">
@@ -5603,7 +5603,7 @@
       </c>
       <c r="B10" s="2" t="inlineStr">
         <is>
-          <t>「当月に計上」＝毎月末にその月分を未払費用に計上（会計基準に沿う。おすすめ）。「納付時」＝翌月末に引き落とされたときに費用にする（簡便な方法）。</t>
+          <t>「当月に計上」＝毎月末にその月分を未払費用に計上します（会計基準に沿います。おすすめ）。「納付時」＝翌月末に引き落とされたときに費用にします（簡便な方法）。</t>
         </is>
       </c>
       <c r="C10" s="9" t="n"/>
@@ -5624,7 +5624,7 @@
       </c>
       <c r="B11" s="2" t="inlineStr">
         <is>
-          <t>「毎月見積計上」＝毎月の賃金から見積って未払費用に計上し、年度更新で精算（会計基準に沿う）。「納付時」＝年度更新の納付のときに一度に費用にする（金額が小さいときの簡便な方法）。</t>
+          <t>「毎月見積計上」＝毎月の賃金から見積って未払費用に計上し、年度更新で精算します（会計基準に沿います）。「納付時」＝年度更新の納付のときに一度に費用にします（金額が小さいときの簡便な方法）。</t>
         </is>
       </c>
       <c r="C11" s="9" t="n"/>
@@ -6364,7 +6364,7 @@
         </is>
       </c>
     </row>
-    <row r="3" ht="126" customHeight="1">
+    <row r="3" ht="138" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
           <t>自分で付ける記号。ほかの表でこの人を指すのに使います。例：E01</t>
@@ -6437,7 +6437,7 @@
       </c>
       <c r="O3" s="6" t="inlineStr">
         <is>
-          <t>住民税の納め方。「特別徴収」＝会社が給与から天引き（このときは「住民税」の表に毎月の金額を書く）。「普通徴収」＝本人が自分で納める（会社は引かない）。</t>
+          <t>住民税の納め方。「特別徴収」＝会社が給与から天引きします（このときは「住民税」の表に毎月の金額を書きます）。「普通徴収」＝本人が自分で納めます（会社は引きません）。</t>
         </is>
       </c>
     </row>

</xml_diff>